<commit_message>
fix: ensure results are logged to all rows including empty/duplicate usernames
</commit_message>
<xml_diff>
--- a/Testdata/testdata_signup.xlsx
+++ b/Testdata/testdata_signup.xlsx
@@ -1,16 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
+  <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -22,7 +17,7 @@
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
-      <sz val="11"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -50,9 +45,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -199,6 +194,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -233,6 +229,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -267,20 +264,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -402,7 +395,46 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
@@ -413,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,6 +466,11 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Result_x000d_</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Result</t>
         </is>
       </c>
@@ -454,7 +491,7 @@
           <t>password123</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -476,12 +513,100 @@
           <t>password456</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>user_test_3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>test3@example.com</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>user_test_4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>password456</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>user_test_4</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>test3@example.com</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>password456</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>test3@example.com</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>password456</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: ensure test status is correctly logged as FAIL for invalid data
</commit_message>
<xml_diff>
--- a/Testdata/testdata_signup.xlsx
+++ b/Testdata/testdata_signup.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,11 +466,6 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Result_x000d_</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
           <t>Result</t>
         </is>
       </c>
@@ -491,7 +486,7 @@
           <t>password123</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -513,7 +508,7 @@
           <t>password456</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -530,9 +525,9 @@
           <t>test3@example.com</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -547,9 +542,9 @@
           <t>password456</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -559,9 +554,9 @@
           <t>user_test_4</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -571,9 +566,9 @@
           <t>test3@example.com</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -583,9 +578,9 @@
           <t>password456</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -600,9 +595,9 @@
           <t>password456</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: expand sign-up test scenarios to cover all cases
</commit_message>
<xml_diff>
--- a/Testdata/testdata_signup.xlsx
+++ b/Testdata/testdata_signup.xlsx
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>user_test_1</t>
+          <t>user_234359</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>test1@example.com</t>
+          <t>user_234359@example.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>password123</t>
+          <t>pass123456</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -495,17 +495,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>user_test_2</t>
+          <t>ผู้ใช้_234359</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>test2@example.com</t>
+          <t>thai_234359@example.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>password456</t>
+          <t>pass123456</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -517,29 +517,34 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>user_test_3</t>
+          <t>spec_234359</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>test3@example.com</t>
+          <t>spec_234359@example.com</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>pass!@#$%^&amp;*()</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>user_test_4</t>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>no_user_234359@example.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>password456</t>
+          <t>pass123456</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -551,7 +556,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>user_test_4</t>
+          <t>no_email_234359</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>pass123456</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -561,9 +571,14 @@
       </c>
     </row>
     <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>no_pass_234359</t>
+        </is>
+      </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>test3@example.com</t>
+          <t>nopass_234359@example.com</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -573,31 +588,46 @@
       </c>
     </row>
     <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>bad_mail_234359</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>not-an-email</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>password456</t>
+          <t>pass123456</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
     </row>
     <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>dup_mail_234359</t>
+        </is>
+      </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>test3@example.com</t>
+          <t>full@example.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>password456</t>
+          <t>pass123456</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
     </row>

</xml_diff>